<commit_message>
Oracle Test Data & Customer Intelligence
</commit_message>
<xml_diff>
--- a/data/processed/Low_Stock_Report.xlsx
+++ b/data/processed/Low_Stock_Report.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -493,161 +493,161 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Potatoes</t>
+          <t>55 Gallon Industrial Trash Bags Case</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Guntur Branch</t>
+          <t>Mock Distribution Branch - Irving</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>3.571428571428572</v>
+        <v>9.714285714285714</v>
       </c>
       <c r="E2" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Potatoes in Guntur Branch inventory is critically low and may run out within the next day based on recent demand patterns. Hyderabad Central can support with 20 surplus units before procurement.</t>
+          <t>55 Gallon Industrial Trash Bags Case in Mock Distribution Branch - Irving is high with stable. Mock Distribution Branch - Chicago can support with 49 surplus units before procurement.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bananas</t>
+          <t>Pallet Stretch Film Case</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hyderabad Central</t>
+          <t>Mock Distribution Branch - Eden Prairie</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>1.08695652173913</v>
+        <v>5.571428571428571</v>
       </c>
       <c r="E3" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Bananas in Hyderabad Central inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Vijayawada Branch can support with 5 surplus units before procurement.</t>
+          <t>Pallet Stretch Film Case in Mock Distribution Branch - Eden Prairie is high with rising. Mock Distribution Branch - Plano can support with 28 surplus units before procurement.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Apples</t>
+          <t>Nitrile Gloves Medium Case</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hyderabad Central</t>
+          <t>Mock Distribution Branch - Dallas</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>41.28571428571428</v>
       </c>
       <c r="E4" t="n">
-        <v>999</v>
+        <v>0.1</v>
       </c>
       <c r="F4" t="n">
-        <v>29</v>
+        <v>269</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Apples in Hyderabad Central needs review because sales history is limited and stock is at or below its reorder point. Vijayawada Branch can support with 5 surplus units before procurement.</t>
+          <t>Nitrile Gloves Medium Case in Mock Distribution Branch - Dallas inventory is critically low and may run out within the next day based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 79 surplus units before procurement.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tomatoes</t>
+          <t>Pallet Stretch Film Case</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Guntur Branch</t>
+          <t>Mock Distribution Branch - Chicago</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="E5" t="n">
-        <v>999</v>
+        <v>0.36</v>
       </c>
       <c r="F5" t="n">
-        <v>14</v>
+        <v>146</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Tomatoes in Guntur Branch needs review because sales history is limited and stock is at or below its reorder point. Hyderabad Central can support with 4 surplus units before procurement.</t>
+          <t>Pallet Stretch Film Case in Mock Distribution Branch - Chicago inventory is critically low and may run out within the next day based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Plano can support with 63 surplus units before procurement.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tomatoes</t>
+          <t>Compostable Takeout Containers Case</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Vijayawada Branch</t>
+          <t>Mock Distribution Branch - Plano</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>8.285714285714286</v>
       </c>
       <c r="E6" t="n">
-        <v>999</v>
+        <v>0.72</v>
       </c>
       <c r="F6" t="n">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Tomatoes in Vijayawada Branch needs review because sales history is limited and stock is at or below its reorder point. Hyderabad Central can support with 2 surplus units before procurement.</t>
+          <t>Compostable Takeout Containers Case in Mock Distribution Branch - Plano inventory is critically low and may run out within the next day based on recent demand patterns. Mock Distribution Branch - Eden Prairie can support with 36 surplus units before procurement.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ice Cream</t>
+          <t>9 inch Paper Plates Case</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Guntur Branch</t>
+          <t>Mock Distribution Branch - Dallas</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -656,27 +656,27 @@
         <v>999</v>
       </c>
       <c r="F7" t="n">
-        <v>11</v>
+        <v>80</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Ice Cream in Guntur Branch needs review because sales history is limited and stock is at or below its reorder point. Hyderabad Central can support with 1 surplus units before procurement.</t>
+          <t>9 inch Paper Plates Case in Mock Distribution Branch - Dallas needs review because sales history is limited and stock is at or below its reorder point. Mock Distribution Branch - Chicago can support with 40 surplus units before procurement.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bananas</t>
+          <t>Disposable Face Masks Case</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Guntur Branch</t>
+          <t>Mock Distribution Branch - Irving</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -685,11 +685,69 @@
         <v>999</v>
       </c>
       <c r="F8" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Bananas in Guntur Branch needs review because sales history is limited and stock is at or below its reorder point. Vijayawada Branch can support with 5 surplus units before procurement.</t>
+          <t>Disposable Face Masks Case in Mock Distribution Branch - Irving needs review because sales history is limited and stock is at or below its reorder point. Mock Distribution Branch - Dallas can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Dallas</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>60</v>
+      </c>
+      <c r="D9" t="n">
+        <v>13.57142857142857</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="F9" t="n">
+        <v>89</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case in Mock Distribution Branch - Dallas inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Mock Distribution Branch - Chicago can support with 8 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Hardwound Paper Towels Case</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Eden Prairie</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>999</v>
+      </c>
+      <c r="F10" t="n">
+        <v>54</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Hardwound Paper Towels Case in Mock Distribution Branch - Eden Prairie needs review because sales history is limited and stock is at or below its reorder point. Mock Distribution Branch - Irving can support with 24 surplus units before procurement.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: Order Simulation & Abnormal Orde Alert Mail
</commit_message>
<xml_diff>
--- a/data/processed/Low_Stock_Report.xlsx
+++ b/data/processed/Low_Stock_Report.xlsx
@@ -441,16 +441,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,20 +473,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Reorder Point</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Inventory Position</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Avg Daily Sales</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Depletion Window (Days)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Suggested Reorder Qty</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>AI Reasoning</t>
         </is>
@@ -493,261 +505,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>55 Gallon Industrial Trash Bags Case</t>
+          <t>Copy Paper Case</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mock Distribution Branch - Irving</t>
+          <t>Network-wide inventory</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="D2" t="n">
-        <v>9.714285714285714</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>64</v>
+        <v>100</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Below reorder threshold</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>55 Gallon Industrial Trash Bags Case in Mock Distribution Branch - Irving is high with stable. Mock Distribution Branch - Chicago can support with 49 surplus units before procurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Pallet Stretch Film Case</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Mock Distribution Branch - Eden Prairie</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>5.571428571428571</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>29</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Pallet Stretch Film Case in Mock Distribution Branch - Eden Prairie is high with rising. Mock Distribution Branch - Plano can support with 28 surplus units before procurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Nitrile Gloves Medium Case</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Mock Distribution Branch - Dallas</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" t="n">
-        <v>41.28571428571428</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F4" t="n">
-        <v>269</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Nitrile Gloves Medium Case in Mock Distribution Branch - Dallas inventory is critically low and may run out within the next day based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 79 surplus units before procurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Pallet Stretch Film Case</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Mock Distribution Branch - Chicago</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D5" t="n">
-        <v>28</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="F5" t="n">
-        <v>146</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Pallet Stretch Film Case in Mock Distribution Branch - Chicago inventory is critically low and may run out within the next day based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Plano can support with 63 surplus units before procurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Compostable Takeout Containers Case</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Mock Distribution Branch - Plano</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D6" t="n">
-        <v>8.285714285714286</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="F6" t="n">
-        <v>44</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Compostable Takeout Containers Case in Mock Distribution Branch - Plano inventory is critically low and may run out within the next day based on recent demand patterns. Mock Distribution Branch - Eden Prairie can support with 36 surplus units before procurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>9 inch Paper Plates Case</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Mock Distribution Branch - Dallas</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>999</v>
-      </c>
-      <c r="F7" t="n">
-        <v>80</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>9 inch Paper Plates Case in Mock Distribution Branch - Dallas needs review because sales history is limited and stock is at or below its reorder point. Mock Distribution Branch - Chicago can support with 40 surplus units before procurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Disposable Face Masks Case</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Mock Distribution Branch - Irving</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>999</v>
-      </c>
-      <c r="F8" t="n">
-        <v>50</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Disposable Face Masks Case in Mock Distribution Branch - Irving needs review because sales history is limited and stock is at or below its reorder point. Mock Distribution Branch - Dallas can support with 25 surplus units before procurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>55 Gallon Industrial Trash Bags Case</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Mock Distribution Branch - Dallas</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>60</v>
-      </c>
-      <c r="D9" t="n">
-        <v>13.57142857142857</v>
-      </c>
-      <c r="E9" t="n">
-        <v>4.42</v>
-      </c>
-      <c r="F9" t="n">
-        <v>89</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>55 Gallon Industrial Trash Bags Case in Mock Distribution Branch - Dallas inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Mock Distribution Branch - Chicago can support with 8 surplus units before procurement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Hardwound Paper Towels Case</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Mock Distribution Branch - Eden Prairie</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>6</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>999</v>
-      </c>
-      <c r="F10" t="n">
-        <v>54</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Hardwound Paper Towels Case in Mock Distribution Branch - Eden Prairie needs review because sales history is limited and stock is at or below its reorder point. Mock Distribution Branch - Irving can support with 24 surplus units before procurement.</t>
+          <t>No recent demand</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>120</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Inventory has fallen below the reorder point of 100 units after order ORD-20260623-9043, leaving 80 units on hand. Initiate replenishment now (suggested ~120 units) to rebuild the safety buffer before further demand creates stockout risk.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Test: Final Smoke Test
</commit_message>
<xml_diff>
--- a/data/processed/Low_Stock_Report.xlsx
+++ b/data/processed/Low_Stock_Report.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -505,19 +505,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Safety Glasses Pack</t>
+          <t>55 Gallon Industrial Trash Bags Case</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Network-wide inventory</t>
+          <t>Mock Distribution Branch - Irving</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>125</v>
+        <v>30</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -526,20 +526,1127 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Less than 1 day remaining</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>16.29/day</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>106</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case in Mock Distribution Branch - Irving is critical with demand spike. Demand spike detected. Mock Distribution Branch - Chicago can support with 49 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Eden Prairie</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Less than 1 day remaining</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>8.43/day</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>44</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case in Mock Distribution Branch - Eden Prairie is critical with demand spike. Demand spike detected. Mock Distribution Branch - Plano can support with 43 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Dallas</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Less than 1 day remaining</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>45.71/day</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>298</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case in Mock Distribution Branch - Dallas inventory is critically low and may run out within the next day based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 63 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Chicago</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Less than 1 day remaining</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>32.00/day</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>167</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case in Mock Distribution Branch - Chicago inventory is critically low and may run out within the next day based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Plano can support with 44 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Plano</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Less than 1 day remaining</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>15.14/day</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>79</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case in Mock Distribution Branch - Plano inventory is critically low and may run out within the next day based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 70 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Dallas</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D7" t="n">
+        <v>30</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2–5 days remaining</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>23.00/day</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>150</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case in Mock Distribution Branch - Dallas inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Chicago can support with 49 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Chicago</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>127</v>
+      </c>
+      <c r="D8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2–5 days remaining</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>34.71/day</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>226</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case in Mock Distribution Branch - Chicago inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Irving can support with 47 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Dallas</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>65</v>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2–5 days remaining</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>17.57/day</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>92</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case in Mock Distribution Branch - Dallas inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 23 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Plano</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>122</v>
+      </c>
+      <c r="D10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2–5 days remaining</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>30.86/day</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>201</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case in Mock Distribution Branch - Plano inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Irving can support with 33 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Plano</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>83</v>
+      </c>
+      <c r="D11" t="n">
+        <v>30</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2–5 days remaining</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>19.57/day</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>128</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case in Mock Distribution Branch - Plano inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Chicago can support with 15 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Eden Prairie</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>119</v>
+      </c>
+      <c r="D12" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2–5 days remaining</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>25.00/day</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>163</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case in Mock Distribution Branch - Eden Prairie inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Irving can support with 6 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Irving</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>49</v>
+      </c>
+      <c r="D13" t="n">
+        <v>25</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2–5 days remaining</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>9.86/day</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>52</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case in Mock Distribution Branch - Irving inventory is at high risk and may deplete within 2–5 days based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Plano can support with 1 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Chicago</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>71</v>
+      </c>
+      <c r="D14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Less than 10 days remaining</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>14.14/day</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>74</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case in Mock Distribution Branch - Chicago inventory needs monitoring with less than 10 days remaining. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Dallas</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>198</v>
+      </c>
+      <c r="D15" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Less than 10 days remaining</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>35.43/day</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>231</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case in Mock Distribution Branch - Dallas inventory needs monitoring with less than 10 days remaining. Demand spike detected. Mock Distribution Branch - Irving can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Irving</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>65</v>
+      </c>
+      <c r="D16" t="n">
+        <v>40</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Less than 10 days remaining</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>10.29/day</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>54</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case in Mock Distribution Branch - Irving inventory needs monitoring with less than 10 days remaining. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>9 inch Paper Plates Case</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Dallas</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Out of stock</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>No recent demand</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>80</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>9 inch Paper Plates Case in Mock Distribution Branch - Dallas needs review because sales history is limited and stock is at or below its reorder point. Mock Distribution Branch - Chicago can support with 40 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Disposable Face Masks Case</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Irving</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>25</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Out of stock</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>No recent demand</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>50</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Disposable Face Masks Case in Mock Distribution Branch - Irving needs review because sales history is limited and stock is at or below its reorder point. Mock Distribution Branch - Dallas can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Eden Prairie</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>98</v>
+      </c>
+      <c r="D19" t="n">
+        <v>30</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Less than 10 days remaining</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>14.14/day</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>92</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case in Mock Distribution Branch - Eden Prairie inventory needs monitoring with less than 10 days remaining. Demand spike detected. Mock Distribution Branch - Chicago can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Dallas</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>82</v>
+      </c>
+      <c r="D20" t="n">
+        <v>25</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Less than 10 days remaining</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>11.29/day</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>59</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case in Mock Distribution Branch - Dallas inventory needs monitoring with less than 10 days remaining. Demand spike detected. Mock Distribution Branch - Plano can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Chicago</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>150</v>
+      </c>
+      <c r="D21" t="n">
+        <v>30</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Less than 10 days remaining</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>20.29/day</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>132</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>55 Gallon Industrial Trash Bags Case in Mock Distribution Branch - Chicago inventory needs monitoring with less than 10 days remaining. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Irving</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>206</v>
+      </c>
+      <c r="D22" t="n">
+        <v>40</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Less than 10 days remaining</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>27.14/day</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>177</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>12 oz Paper Hot Cups Case in Mock Distribution Branch - Irving inventory needs monitoring with less than 10 days remaining. Demand spike detected. Mock Distribution Branch - Dallas can support with 21 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Chicago</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>99</v>
+      </c>
+      <c r="D23" t="n">
+        <v>25</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Less than 10 days remaining</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>11.86/day</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>78</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case in Mock Distribution Branch - Chicago inventory needs monitoring with less than 10 days remaining. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Plano</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>95</v>
+      </c>
+      <c r="D24" t="n">
+        <v>25</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Less than 10 days remaining</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>10.29/day</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>54</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Pallet Stretch Film Case in Mock Distribution Branch - Plano inventory needs monitoring with less than 10 days remaining. Demand spike detected. Mock Distribution Branch - Dallas can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Plano</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>109</v>
+      </c>
+      <c r="D25" t="n">
+        <v>25</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Healthy</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2–4 weeks remaining</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>10.86/day</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>71</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case in Mock Distribution Branch - Plano inventory is stable based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Irving</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>108</v>
+      </c>
+      <c r="D26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Healthy</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2–4 weeks remaining</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>10.00/day</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>65</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case in Mock Distribution Branch - Irving inventory is stable based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Eden Prairie can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Eden Prairie</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>104</v>
+      </c>
+      <c r="D27" t="n">
+        <v>25</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Healthy</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2–4 weeks remaining</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>8.29/day</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>54</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Nitrile Gloves Medium Case in Mock Distribution Branch - Eden Prairie inventory is stable based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Irving can support with 25 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Eden Prairie</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>205</v>
+      </c>
+      <c r="D28" t="n">
+        <v>40</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Healthy</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2–4 weeks remaining</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>11.57/day</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>61</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Compostable Takeout Containers Case in Mock Distribution Branch - Eden Prairie inventory is stable based on recent demand patterns. Demand spike detected. Mock Distribution Branch - Irving can support with 14 surplus units before procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Hardwound Paper Towels Case</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Mock Distribution Branch - Eden Prairie</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>30</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>Below reorder threshold</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>No recent demand</t>
         </is>
       </c>
-      <c r="H2" t="n">
-        <v>140</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Inventory has fallen below the reorder point of 125 units after order ORD-20260623-9046, leaving 110 units on hand. Initiate replenishment now (suggested ~140 units) to rebuild the safety buffer before further demand creates stockout risk.</t>
+      <c r="H29" t="n">
+        <v>54</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Hardwound Paper Towels Case in Mock Distribution Branch - Eden Prairie needs review because sales history is limited and stock is at or below its reorder point. Mock Distribution Branch - Irving can support with 24 surplus units before procurement.</t>
         </is>
       </c>
     </row>

</xml_diff>